<commit_message>
make warnings in tests disappear (because of clashing value label of value 1 when using powerjoin)
</commit_message>
<xml_diff>
--- a/tests/testthat/excel/mapping_old.xlsx
+++ b/tests/testthat/excel/mapping_old.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="26026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="26529"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="K:\Projects\UW git\datenanpassr\tests\testthat\excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{F30B4BA8-C1A2-4D2E-B652-B9E8004B6A08}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F96A68F7-6F65-4146-87A9-CD73EC5BC738}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="14250" tabRatio="500" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15525" tabRatio="500" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="configr" sheetId="1" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="286" uniqueCount="187">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="286" uniqueCount="186">
   <si>
     <t>item</t>
   </si>
@@ -494,9 +494,6 @@
   </si>
   <si>
     <t>#MERGE</t>
-  </si>
-  <si>
-    <t>q1 q2</t>
   </si>
   <si>
     <t>#RFUN</t>
@@ -1625,7 +1622,7 @@
         <v>113</v>
       </c>
       <c r="B5" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="C5">
         <v>10</v>
@@ -1636,7 +1633,7 @@
         <v>113</v>
       </c>
       <c r="B6" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="C6">
         <v>11</v>
@@ -1894,10 +1891,10 @@
         <v>105</v>
       </c>
       <c r="H24" s="2" t="s">
+        <v>161</v>
+      </c>
+      <c r="T24" t="s">
         <v>162</v>
-      </c>
-      <c r="T24" t="s">
-        <v>163</v>
       </c>
     </row>
   </sheetData>
@@ -2021,7 +2018,7 @@
         <v>3</v>
       </c>
       <c r="E11" s="6" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.25">
@@ -2035,7 +2032,7 @@
         <v>3</v>
       </c>
       <c r="E12" s="6" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.25">
@@ -2133,7 +2130,7 @@
         <v>130</v>
       </c>
       <c r="B27" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="C27" t="s">
         <v>140</v>
@@ -2208,61 +2205,61 @@
         <v>151</v>
       </c>
       <c r="B38" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="C38" t="s">
         <v>4</v>
       </c>
       <c r="D38" t="s">
-        <v>152</v>
+        <v>24</v>
       </c>
     </row>
     <row r="40" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
+        <v>152</v>
+      </c>
+      <c r="B40" t="s">
         <v>153</v>
       </c>
-      <c r="B40" t="s">
+      <c r="C40" t="s">
         <v>154</v>
-      </c>
-      <c r="C40" t="s">
-        <v>155</v>
       </c>
     </row>
     <row r="41" spans="1:7" x14ac:dyDescent="0.25">
       <c r="F41" s="7" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
     </row>
     <row r="42" spans="1:7" x14ac:dyDescent="0.25">
       <c r="F42" s="7" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="G42" s="7" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
     </row>
     <row r="43" spans="1:7" x14ac:dyDescent="0.25">
       <c r="F43" s="7"/>
       <c r="G43" s="7" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
     </row>
     <row r="44" spans="1:7" x14ac:dyDescent="0.25">
       <c r="F44" s="7"/>
       <c r="G44" s="7" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
     </row>
     <row r="45" spans="1:7" x14ac:dyDescent="0.25">
       <c r="F45" s="7"/>
       <c r="G45" s="7" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
     </row>
     <row r="46" spans="1:7" x14ac:dyDescent="0.25">
       <c r="F46" s="7"/>
       <c r="G46" s="7" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
     </row>
     <row r="48" spans="1:7" x14ac:dyDescent="0.25">
@@ -2270,13 +2267,13 @@
         <v>121</v>
       </c>
       <c r="B48" t="s">
+        <v>156</v>
+      </c>
+      <c r="C48" t="s">
         <v>157</v>
       </c>
-      <c r="C48" t="s">
+      <c r="D48" t="s">
         <v>158</v>
-      </c>
-      <c r="D48" t="s">
-        <v>159</v>
       </c>
     </row>
     <row r="49" spans="1:5" x14ac:dyDescent="0.25">
@@ -2298,7 +2295,7 @@
         <v>2</v>
       </c>
       <c r="E50" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
     </row>
     <row r="51" spans="1:5" x14ac:dyDescent="0.25">
@@ -2327,7 +2324,7 @@
     </row>
     <row r="56" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="B56" t="s">
         <v>24</v>
@@ -2336,7 +2333,7 @@
         <v>24</v>
       </c>
       <c r="D56" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
     </row>
     <row r="57" spans="1:5" x14ac:dyDescent="0.25">
@@ -2346,13 +2343,13 @@
     </row>
     <row r="59" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="B59" t="s">
         <v>31</v>
       </c>
       <c r="C59" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
     </row>
     <row r="60" spans="1:5" x14ac:dyDescent="0.25">
@@ -2360,25 +2357,25 @@
         <v>36</v>
       </c>
       <c r="C60" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
     </row>
     <row r="62" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="B62" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
     </row>
     <row r="63" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B63" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
     </row>
     <row r="64" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B64" s="8" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
     </row>
     <row r="65" spans="1:2" x14ac:dyDescent="0.25">
@@ -2386,15 +2383,15 @@
     </row>
     <row r="66" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
+        <v>182</v>
+      </c>
+      <c r="B66" t="s">
         <v>183</v>
-      </c>
-      <c r="B66" t="s">
-        <v>184</v>
       </c>
     </row>
     <row r="67" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B67" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
     </row>
   </sheetData>
@@ -2416,7 +2413,7 @@
         <v>113</v>
       </c>
       <c r="B2" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="C2">
         <v>3</v>

</xml_diff>

<commit_message>
add command in line 71 of Free1 sheet that demonstrates refering to dat_mod in #COMP command (silly example: calculate the sum of all variables starting with "q" and followed by 1 digit except q7) (cf. ad8a733233ce03efae54e11a7e181a21921dde92)
</commit_message>
<xml_diff>
--- a/tests/testthat/excel/mapping_old.xlsx
+++ b/tests/testthat/excel/mapping_old.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="K:\Projects\UW git\datenanpassr\tests\testthat\excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F96A68F7-6F65-4146-87A9-CD73EC5BC738}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EF668815-B78E-4E83-A2F3-CA09A10DD20C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15525" tabRatio="500" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="286" uniqueCount="186">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="289" uniqueCount="188">
   <si>
     <t>item</t>
   </si>
@@ -596,6 +596,12 @@
   </si>
   <si>
     <t>../spss/fake_survey.sav</t>
+  </si>
+  <si>
+    <t>qsum</t>
+  </si>
+  <si>
+    <t>rowSums(dat_mod |&gt; dplyr::select(dplyr::matches("^q\\d$"), -q7))</t>
   </si>
 </sst>
 </file>
@@ -1905,7 +1911,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
-  <dimension ref="A1:G67"/>
+  <dimension ref="A1:G71"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.28515625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -2378,10 +2384,10 @@
         <v>179</v>
       </c>
     </row>
-    <row r="65" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B65" s="8"/>
     </row>
-    <row r="66" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
         <v>182</v>
       </c>
@@ -2389,9 +2395,20 @@
         <v>183</v>
       </c>
     </row>
-    <row r="67" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B67" t="s">
         <v>184</v>
+      </c>
+    </row>
+    <row r="71" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A71" t="s">
+        <v>113</v>
+      </c>
+      <c r="B71" t="s">
+        <v>186</v>
+      </c>
+      <c r="C71" t="s">
+        <v>187</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
add optional .names argument in column D
</commit_message>
<xml_diff>
--- a/tests/testthat/excel/mapping_old.xlsx
+++ b/tests/testthat/excel/mapping_old.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="K:\Projects\UW git\datenanpassr\tests\testthat\excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B76C99FB-B8A8-44AB-BA1A-59EAF922340A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FCC33663-18DF-4E17-BD35-A33910919D37}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15045" tabRatio="500" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="293" uniqueCount="192">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="294" uniqueCount="193">
   <si>
     <t>item</t>
   </si>
@@ -608,6 +608,9 @@
   </si>
   <si>
     <t>where(is.numeric)</t>
+  </si>
+  <si>
+    <t>{.col}_2</t>
   </si>
   <si>
     <t>\(x) {x[x == 1] &lt;- NA; attr(x, "labels") &lt;- attr(x, "labels")[attr(x, "labels") != 1]; x}</t>
@@ -2396,10 +2399,10 @@
         <v>179</v>
       </c>
     </row>
-    <row r="65" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B65" s="8"/>
     </row>
-    <row r="66" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
         <v>182</v>
       </c>
@@ -2407,12 +2410,12 @@
         <v>183</v>
       </c>
     </row>
-    <row r="67" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B67" t="s">
         <v>184</v>
       </c>
     </row>
-    <row r="71" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
         <v>113</v>
       </c>
@@ -2423,19 +2426,22 @@
         <v>187</v>
       </c>
     </row>
-    <row r="73" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
         <v>188</v>
       </c>
       <c r="B73" t="s">
-        <v>191</v>
-      </c>
-    </row>
-    <row r="74" spans="1:3" x14ac:dyDescent="0.25">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="74" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B74" t="s">
         <v>189</v>
       </c>
       <c r="C74" t="s">
+        <v>191</v>
+      </c>
+      <c r="D74" t="s">
         <v>190</v>
       </c>
     </row>

</xml_diff>

<commit_message>
- fix: remove NA from empty excel cells (possibly at the bottom of the command block) - allow to pass an unnamed list of multiple functions to the `.fns` argument of dplyr::across()
</commit_message>
<xml_diff>
--- a/tests/testthat/excel/mapping_old.xlsx
+++ b/tests/testthat/excel/mapping_old.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="K:\Projects\UW git\datenanpassr\tests\testthat\excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FCC33663-18DF-4E17-BD35-A33910919D37}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{97EEFBBD-11CB-4B1E-A2F1-936D5E4642CE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15045" tabRatio="500" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="294" uniqueCount="193">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="295" uniqueCount="194">
   <si>
     <t>item</t>
   </si>
@@ -610,13 +610,16 @@
     <t>where(is.numeric)</t>
   </si>
   <si>
-    <t>{.col}_2</t>
-  </si>
-  <si>
     <t>\(x) {x[x == 1] &lt;- NA; attr(x, "labels") &lt;- attr(x, "labels")[attr(x, "labels") != 1]; x}</t>
   </si>
   <si>
     <t>matches("^q[1-2]$")</t>
+  </si>
+  <si>
+    <t>\(x) {x * 2}</t>
+  </si>
+  <si>
+    <t>{.col}_{.fn}b</t>
   </si>
 </sst>
 </file>
@@ -1926,7 +1929,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
-  <dimension ref="A1:G74"/>
+  <dimension ref="A1:G75"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.28515625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -2431,7 +2434,7 @@
         <v>188</v>
       </c>
       <c r="B73" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
     </row>
     <row r="74" spans="1:4" x14ac:dyDescent="0.25">
@@ -2439,9 +2442,14 @@
         <v>189</v>
       </c>
       <c r="C74" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="D74" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="75" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="C75" t="s">
         <v>190</v>
       </c>
     </row>

</xml_diff>

<commit_message>
only read the first row of column B into the .cols argument of dplyr::across()
</commit_message>
<xml_diff>
--- a/tests/testthat/excel/mapping_old.xlsx
+++ b/tests/testthat/excel/mapping_old.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="K:\Projects\UW git\datenanpassr\tests\testthat\excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{97EEFBBD-11CB-4B1E-A2F1-936D5E4642CE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{637AB7AA-1C01-402D-8A44-D2A0921FA2E0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15045" tabRatio="500" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="295" uniqueCount="194">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="294" uniqueCount="193">
   <si>
     <t>item</t>
   </si>
@@ -607,19 +607,16 @@
     <t>#ACROSS</t>
   </si>
   <si>
-    <t>where(is.numeric)</t>
-  </si>
-  <si>
     <t>\(x) {x[x == 1] &lt;- NA; attr(x, "labels") &lt;- attr(x, "labels")[attr(x, "labels") != 1]; x}</t>
   </si>
   <si>
-    <t>matches("^q[1-2]$")</t>
-  </si>
-  <si>
     <t>\(x) {x * 2}</t>
   </si>
   <si>
     <t>{.col}_{.fn}b</t>
+  </si>
+  <si>
+    <t>matches("^q[1-2]$") &amp; where(is.numeric)</t>
   </si>
 </sst>
 </file>
@@ -2434,23 +2431,20 @@
         <v>188</v>
       </c>
       <c r="B73" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="74" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="C74" t="s">
+        <v>190</v>
+      </c>
+      <c r="D74" t="s">
         <v>191</v>
-      </c>
-    </row>
-    <row r="74" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="B74" t="s">
-        <v>189</v>
-      </c>
-      <c r="C74" t="s">
-        <v>192</v>
-      </c>
-      <c r="D74" t="s">
-        <v>193</v>
       </c>
     </row>
     <row r="75" spans="1:4" x14ac:dyDescent="0.25">
       <c r="C75" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
- move .names argument from D2 to C1 in command block - don't curlychop() #ACROSS command blocks
</commit_message>
<xml_diff>
--- a/tests/testthat/excel/mapping_old.xlsx
+++ b/tests/testthat/excel/mapping_old.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="K:\Projects\UW git\datenanpassr\tests\testthat\excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{637AB7AA-1C01-402D-8A44-D2A0921FA2E0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{33987E86-E2F4-4354-8C67-D597FC5C1F60}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15045" tabRatio="500" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2399,10 +2399,10 @@
         <v>179</v>
       </c>
     </row>
-    <row r="65" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B65" s="8"/>
     </row>
-    <row r="66" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
         <v>182</v>
       </c>
@@ -2410,12 +2410,12 @@
         <v>183</v>
       </c>
     </row>
-    <row r="67" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B67" t="s">
         <v>184</v>
       </c>
     </row>
-    <row r="71" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
         <v>113</v>
       </c>
@@ -2426,23 +2426,23 @@
         <v>187</v>
       </c>
     </row>
-    <row r="73" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
         <v>188</v>
       </c>
       <c r="B73" t="s">
         <v>192</v>
       </c>
-    </row>
-    <row r="74" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="C73" t="s">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="74" spans="1:3" x14ac:dyDescent="0.25">
       <c r="C74" t="s">
         <v>190</v>
       </c>
-      <c r="D74" t="s">
-        <v>191</v>
-      </c>
-    </row>
-    <row r="75" spans="1:4" x14ac:dyDescent="0.25">
+    </row>
+    <row r="75" spans="1:3" x14ac:dyDescent="0.25">
       <c r="C75" t="s">
         <v>189</v>
       </c>

</xml_diff>

<commit_message>
add possibility to pass a named list of functions to the `.fns` argument of dplyr::across()
</commit_message>
<xml_diff>
--- a/tests/testthat/excel/mapping_old.xlsx
+++ b/tests/testthat/excel/mapping_old.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="K:\Projects\UW git\datenanpassr\tests\testthat\excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{33987E86-E2F4-4354-8C67-D597FC5C1F60}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{82AA540D-1373-4506-9904-AA27E35B09F4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15045" tabRatio="500" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="294" uniqueCount="193">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="296" uniqueCount="195">
   <si>
     <t>item</t>
   </si>
@@ -613,10 +613,16 @@
     <t>\(x) {x * 2}</t>
   </si>
   <si>
-    <t>{.col}_{.fn}b</t>
-  </si>
-  <si>
     <t>matches("^q[1-2]$") &amp; where(is.numeric)</t>
+  </si>
+  <si>
+    <t>{.col}_{.fn}</t>
+  </si>
+  <si>
+    <t>x2</t>
+  </si>
+  <si>
+    <t>rmval</t>
   </si>
 </sst>
 </file>
@@ -2431,18 +2437,24 @@
         <v>188</v>
       </c>
       <c r="B73" t="s">
+        <v>191</v>
+      </c>
+      <c r="C73" t="s">
         <v>192</v>
       </c>
-      <c r="C73" t="s">
-        <v>191</v>
-      </c>
     </row>
     <row r="74" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B74" t="s">
+        <v>193</v>
+      </c>
       <c r="C74" t="s">
         <v>190</v>
       </c>
     </row>
     <row r="75" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B75" t="s">
+        <v>194</v>
+      </c>
       <c r="C75" t="s">
         <v>189</v>
       </c>

</xml_diff>

<commit_message>
add coal = "xy" to #MERGE example in excel mapping and update snapshots
</commit_message>
<xml_diff>
--- a/tests/testthat/excel/mapping_old.xlsx
+++ b/tests/testthat/excel/mapping_old.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="26626"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24332"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="K:\Projects\UW git\datenanpassr\tests\testthat\excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{82AA540D-1373-4506-9904-AA27E35B09F4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4B544FC3-6D4C-4E45-8DF9-576D194F81A8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15045" tabRatio="500" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="296" uniqueCount="195">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="297" uniqueCount="196">
   <si>
     <t>item</t>
   </si>
@@ -623,6 +623,9 @@
   </si>
   <si>
     <t>rmval</t>
+  </si>
+  <si>
+    <t>xy</t>
   </si>
 </sst>
 </file>
@@ -2240,6 +2243,9 @@
       <c r="D38" t="s">
         <v>24</v>
       </c>
+      <c r="E38" t="s">
+        <v>195</v>
+      </c>
     </row>
     <row r="40" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A40" t="s">

</xml_diff>

<commit_message>
- refactor to use openxlsx2 instead of openxlsx & readxl - store openxlsx2 workbook as a field in the Mapping object and use this for reading in the named regions and the sheets - the verbatims file sheets' content is also read in from the same openxlsx2 workbook object
</commit_message>
<xml_diff>
--- a/tests/testthat/excel/mapping_old.xlsx
+++ b/tests/testthat/excel/mapping_old.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="K:\Projects\UW git\datenanpassr\tests\testthat\excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4B544FC3-6D4C-4E45-8DF9-576D194F81A8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CDA4D752-60E6-440C-B100-B78506B4D9D7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15045" tabRatio="500" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15045" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="configr" sheetId="1" r:id="rId1"/>
@@ -30,6 +30,15 @@
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
     <ext xmlns:loext="http://schemas.libreoffice.org/" uri="{7626C862-2A13-11E5-B345-FEFF819CDC9F}">
       <loext:extCalcPr stringRefSyntax="ExcelA1"/>
     </ext>
@@ -1676,7 +1685,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
-  <dimension ref="B1:T24"/>
+  <dimension ref="B1:T25"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="2:4" x14ac:dyDescent="0.25">
@@ -1734,128 +1743,105 @@
         <v>79</v>
       </c>
     </row>
-    <row r="17" spans="2:20" x14ac:dyDescent="0.25">
-      <c r="B17" t="s">
-        <v>80</v>
-      </c>
-      <c r="C17" t="s">
-        <v>81</v>
-      </c>
-      <c r="D17" t="s">
-        <v>82</v>
-      </c>
-      <c r="E17" t="s">
-        <v>83</v>
-      </c>
-      <c r="F17" t="s">
-        <v>84</v>
-      </c>
-      <c r="G17" t="s">
-        <v>85</v>
-      </c>
-      <c r="H17" t="s">
-        <v>86</v>
-      </c>
-      <c r="I17" t="s">
-        <v>87</v>
-      </c>
-      <c r="J17" t="s">
-        <v>88</v>
-      </c>
-      <c r="K17" t="s">
-        <v>89</v>
-      </c>
-      <c r="L17" t="s">
-        <v>90</v>
-      </c>
-      <c r="M17" t="s">
-        <v>91</v>
-      </c>
-      <c r="N17" t="s">
-        <v>92</v>
-      </c>
-      <c r="O17" t="s">
-        <v>93</v>
-      </c>
-      <c r="P17" t="s">
-        <v>94</v>
-      </c>
-      <c r="Q17" t="s">
-        <v>95</v>
-      </c>
-      <c r="R17" t="s">
-        <v>96</v>
-      </c>
-      <c r="S17" t="s">
-        <v>97</v>
-      </c>
-      <c r="T17" t="s">
-        <v>98</v>
-      </c>
-    </row>
     <row r="18" spans="2:20" x14ac:dyDescent="0.25">
       <c r="B18" t="s">
-        <v>40</v>
-      </c>
-      <c r="C18">
-        <v>1</v>
+        <v>80</v>
+      </c>
+      <c r="C18" t="s">
+        <v>81</v>
       </c>
       <c r="D18" t="s">
-        <v>99</v>
+        <v>82</v>
+      </c>
+      <c r="E18" t="s">
+        <v>83</v>
+      </c>
+      <c r="F18" t="s">
+        <v>84</v>
+      </c>
+      <c r="G18" t="s">
+        <v>85</v>
       </c>
       <c r="H18" t="s">
-        <v>100</v>
+        <v>86</v>
+      </c>
+      <c r="I18" t="s">
+        <v>87</v>
+      </c>
+      <c r="J18" t="s">
+        <v>88</v>
+      </c>
+      <c r="K18" t="s">
+        <v>89</v>
+      </c>
+      <c r="L18" t="s">
+        <v>90</v>
+      </c>
+      <c r="M18" t="s">
+        <v>91</v>
+      </c>
+      <c r="N18" t="s">
+        <v>92</v>
+      </c>
+      <c r="O18" t="s">
+        <v>93</v>
+      </c>
+      <c r="P18" t="s">
+        <v>94</v>
+      </c>
+      <c r="Q18" t="s">
+        <v>95</v>
       </c>
       <c r="R18" t="s">
-        <v>99</v>
+        <v>96</v>
       </c>
       <c r="S18" t="s">
-        <v>101</v>
+        <v>97</v>
+      </c>
+      <c r="T18" t="s">
+        <v>98</v>
       </c>
     </row>
     <row r="19" spans="2:20" x14ac:dyDescent="0.25">
       <c r="B19" t="s">
-        <v>102</v>
+        <v>40</v>
       </c>
       <c r="C19">
         <v>1</v>
       </c>
       <c r="D19" t="s">
+        <v>99</v>
+      </c>
+      <c r="H19" t="s">
+        <v>100</v>
+      </c>
+      <c r="R19" t="s">
+        <v>99</v>
+      </c>
+      <c r="S19" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="20" spans="2:20" x14ac:dyDescent="0.25">
+      <c r="B20" t="s">
+        <v>102</v>
+      </c>
+      <c r="C20">
+        <v>1</v>
+      </c>
+      <c r="D20" t="s">
         <v>103</v>
       </c>
-      <c r="H19" t="s">
+      <c r="H20" t="s">
         <v>104</v>
       </c>
-      <c r="R19" t="s">
+      <c r="R20" t="s">
         <v>103</v>
-      </c>
-    </row>
-    <row r="20" spans="2:20" x14ac:dyDescent="0.25">
-      <c r="B20" s="2" t="s">
-        <v>40</v>
-      </c>
-      <c r="C20" s="2">
-        <v>3</v>
-      </c>
-      <c r="D20" s="2" t="s">
-        <v>105</v>
-      </c>
-      <c r="E20" s="2"/>
-      <c r="F20" s="2"/>
-      <c r="G20" s="2"/>
-      <c r="H20" s="2" t="s">
-        <v>106</v>
-      </c>
-      <c r="I20" s="2"/>
-      <c r="J20" s="2"/>
-      <c r="K20" s="2"/>
-      <c r="L20" s="2">
-        <v>100</v>
       </c>
     </row>
     <row r="21" spans="2:20" x14ac:dyDescent="0.25">
       <c r="B21" s="2" t="s">
-        <v>107</v>
+        <v>40</v>
       </c>
       <c r="C21" s="2">
         <v>3</v>
@@ -1867,7 +1853,7 @@
       <c r="F21" s="2"/>
       <c r="G21" s="2"/>
       <c r="H21" s="2" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="I21" s="2"/>
       <c r="J21" s="2"/>
@@ -1877,19 +1863,25 @@
       </c>
     </row>
     <row r="22" spans="2:20" x14ac:dyDescent="0.25">
-      <c r="B22" t="s">
-        <v>40</v>
-      </c>
-      <c r="C22">
-        <v>2</v>
-      </c>
-      <c r="D22" t="s">
-        <v>109</v>
-      </c>
-      <c r="H22" t="s">
-        <v>110</v>
-      </c>
-      <c r="L22">
+      <c r="B22" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="C22" s="2">
+        <v>3</v>
+      </c>
+      <c r="D22" s="2" t="s">
+        <v>105</v>
+      </c>
+      <c r="E22" s="2"/>
+      <c r="F22" s="2"/>
+      <c r="G22" s="2"/>
+      <c r="H22" s="2" t="s">
+        <v>108</v>
+      </c>
+      <c r="I22" s="2"/>
+      <c r="J22" s="2"/>
+      <c r="K22" s="2"/>
+      <c r="L22" s="2">
         <v>100</v>
       </c>
     </row>
@@ -1897,17 +1889,17 @@
       <c r="B23" t="s">
         <v>40</v>
       </c>
-      <c r="C23" t="s">
-        <v>111</v>
+      <c r="C23">
+        <v>2</v>
       </c>
       <c r="D23" t="s">
-        <v>105</v>
-      </c>
-      <c r="H23" s="2" t="s">
-        <v>112</v>
-      </c>
-      <c r="T23" t="s">
-        <v>24</v>
+        <v>109</v>
+      </c>
+      <c r="H23" t="s">
+        <v>110</v>
+      </c>
+      <c r="L23">
+        <v>100</v>
       </c>
     </row>
     <row r="24" spans="2:20" x14ac:dyDescent="0.25">
@@ -1921,9 +1913,26 @@
         <v>105</v>
       </c>
       <c r="H24" s="2" t="s">
+        <v>112</v>
+      </c>
+      <c r="T24" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="25" spans="2:20" x14ac:dyDescent="0.25">
+      <c r="B25" t="s">
+        <v>40</v>
+      </c>
+      <c r="C25" t="s">
+        <v>111</v>
+      </c>
+      <c r="D25" t="s">
+        <v>105</v>
+      </c>
+      <c r="H25" s="2" t="s">
         <v>161</v>
       </c>
-      <c r="T24" t="s">
+      <c r="T25" t="s">
         <v>162</v>
       </c>
     </row>

</xml_diff>

<commit_message>
add an unlabelled value in #REC command
</commit_message>
<xml_diff>
--- a/tests/testthat/excel/mapping_old.xlsx
+++ b/tests/testthat/excel/mapping_old.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="K:\Projects\UW git\datenanpassr\tests\testthat\excel\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="K:\Projects\UW git\datadaptor\tests\testthat\excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CDA4D752-60E6-440C-B100-B78506B4D9D7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9DA71264-A646-4A30-A383-9B43099ACE99}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15045" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15525" tabRatio="500" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="configr" sheetId="1" r:id="rId1"/>
@@ -2361,7 +2361,7 @@
         <v>5</v>
       </c>
       <c r="D53">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="56" spans="1:5" x14ac:dyDescent="0.25">

</xml_diff>